<commit_message>
Add Workday official scraper
</commit_message>
<xml_diff>
--- a/data/company_database.xlsx
+++ b/data/company_database.xlsx
@@ -1020,7 +1020,7 @@
       <c r="V3" s="12" t="str"/>
       <c r="W3" s="12" t="inlineStr">
         <is>
-          <t>High fit for Process Support Engineer / Customer Engineer new grad roles; ATS imported from internships; scraper not active for workday</t>
+          <t>High fit for Process Support Engineer / Customer Engineer new grad roles; ATS imported from internships; scraper not active for workday; Workday scraper enabled</t>
         </is>
       </c>
       <c r="X3" s="12" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
@@ -1667,7 +1667,7 @@
       <c r="V9" s="12" t="str"/>
       <c r="W9" s="12" t="inlineStr">
         <is>
-          <t>ATS imported from internships; scraper not active for workday</t>
+          <t>ATS imported from internships; scraper not active for workday; Workday scraper enabled</t>
         </is>
       </c>
       <c r="X9" s="12" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
@@ -1802,7 +1802,7 @@
       <c r="V10" s="12" t="str"/>
       <c r="W10" s="12" t="inlineStr">
         <is>
-          <t>ATS imported from new-grad; scraper not active for workday</t>
+          <t>ATS imported from new-grad; scraper not active for workday; Workday scraper enabled</t>
         </is>
       </c>
       <c r="X10" s="12" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
@@ -1937,7 +1937,7 @@
       <c r="V11" s="12" t="str"/>
       <c r="W11" s="12" t="inlineStr">
         <is>
-          <t>ATS imported from new-grad; scraper not active for workday</t>
+          <t>ATS imported from new-grad; scraper not active for workday; Workday scraper enabled</t>
         </is>
       </c>
       <c r="X11" s="12" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
@@ -3435,7 +3435,7 @@
       <c r="V25" s="12" t="str"/>
       <c r="W25" s="12" t="inlineStr">
         <is>
-          <t>ATS imported from new-grad; scraper not active for workday</t>
+          <t>ATS imported from new-grad; scraper not active for workday; Workday scraper enabled</t>
         </is>
       </c>
       <c r="X25" s="12" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE25" t="inlineStr">
@@ -4837,7 +4837,7 @@
       <c r="V38" s="12" t="str"/>
       <c r="W38" s="12" t="inlineStr">
         <is>
-          <t>ATS imported from new-grad; scraper not active for workday; ATS imported from internships; scraper not active for workday</t>
+          <t>ATS imported from new-grad; scraper not active for workday; ATS imported from internships; scraper not active for workday; Workday scraper enabled</t>
         </is>
       </c>
       <c r="X38" s="12" t="inlineStr">
@@ -4870,7 +4870,7 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="AE38" t="inlineStr">

</xml_diff>